<commit_message>
correcting labels impacto renda gastos
</commit_message>
<xml_diff>
--- a/output/elasticidades.xlsx
+++ b/output/elasticidades.xlsx
@@ -1,21 +1,110 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\tarifas_setor_eletrico\output\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{226FC8F3-64CE-426F-A65F-43B1AF41984D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+  <si>
+    <t>grupo</t>
+  </si>
+  <si>
+    <t>elasticidade</t>
+  </si>
+  <si>
+    <t>se</t>
+  </si>
+  <si>
+    <t>ic_inf</t>
+  </si>
+  <si>
+    <t>ic_sup</t>
+  </si>
+  <si>
+    <t>grupo_label</t>
+  </si>
+  <si>
+    <t>mulher_negra_renda_media</t>
+  </si>
+  <si>
+    <t>Mulher negra (renda média)</t>
+  </si>
+  <si>
+    <t>mulher_negra_renda_alta</t>
+  </si>
+  <si>
+    <t>Mulher negra (renda alta)</t>
+  </si>
+  <si>
+    <t>homem_branco_renda_media</t>
+  </si>
+  <si>
+    <t>Homem branco (renda média)</t>
+  </si>
+  <si>
+    <t>homem_branco_renda_alta</t>
+  </si>
+  <si>
+    <t>Homem branco (renda alta)</t>
+  </si>
+  <si>
+    <t>mulher_branca_renda_media</t>
+  </si>
+  <si>
+    <t>Mulher branca (renda média)</t>
+  </si>
+  <si>
+    <t>mulher_branca_renda_alta</t>
+  </si>
+  <si>
+    <t>Mulher branca (renda alta)</t>
+  </si>
+  <si>
+    <t>homem_negro_renda_alta</t>
+  </si>
+  <si>
+    <t>Homem negro (renda alta)</t>
+  </si>
+  <si>
+    <t>homem_negro_renda_media</t>
+  </si>
+  <si>
+    <t>Homem negro (renda média)</t>
+  </si>
+  <si>
+    <t>rural</t>
+  </si>
+  <si>
+    <t>Zona rural</t>
+  </si>
+  <si>
+    <t>urbano</t>
+  </si>
+  <si>
+    <t>Zona urbana</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -52,24 +141,33 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -107,7 +205,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -141,6 +239,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -175,9 +274,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -350,184 +450,234 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F7"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:F11"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="26.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.26953125" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="13" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>grupo</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>elasticidade</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>se</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>ic_inf</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>ic_sup</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>grupo_label</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>mulher_negra_renda_media</t>
-        </is>
-      </c>
-      <c r="B2">
-        <v>-0.1468246252333343</v>
-      </c>
-      <c r="C2">
-        <v>0.02667335101783406</v>
-      </c>
-      <c r="D2">
+    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="2">
+        <v>-0.14682462523333431</v>
+      </c>
+      <c r="C2" s="2">
+        <v>2.6673351017834059E-2</v>
+      </c>
+      <c r="D2" s="2">
         <v>-0.1991043932282891</v>
       </c>
-      <c r="E2">
-        <v>-0.09454485723837958</v>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Mulher negra (renda média)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>homem_branco_renda_media</t>
-        </is>
-      </c>
-      <c r="B3">
-        <v>-0.3386897463556213</v>
-      </c>
-      <c r="C3">
-        <v>0.036356979251561</v>
-      </c>
-      <c r="D3">
-        <v>-0.4099494256886808</v>
-      </c>
-      <c r="E3">
-        <v>-0.2674300670225617</v>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Homem branco (renda média)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>homem_branco_renda_alta</t>
-        </is>
-      </c>
-      <c r="B4">
-        <v>-0.400538446112141</v>
-      </c>
-      <c r="C4">
-        <v>0.06204813025641015</v>
-      </c>
-      <c r="D4">
-        <v>-0.5221527814147049</v>
-      </c>
-      <c r="E4">
-        <v>-0.2789241108095771</v>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Homem branco (renda alta)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>mulher_branca_renda_alta</t>
-        </is>
-      </c>
-      <c r="B5">
-        <v>-0.3514182688986457</v>
-      </c>
-      <c r="C5">
-        <v>0.09034248415583285</v>
-      </c>
-      <c r="D5">
-        <v>-0.528489537844078</v>
-      </c>
-      <c r="E5">
-        <v>-0.1743469999532133</v>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Mulher branca (renda alta)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>rural</t>
-        </is>
-      </c>
-      <c r="B6">
-        <v>-0.2788930944572934</v>
-      </c>
-      <c r="C6">
-        <v>0.03340928071244035</v>
-      </c>
-      <c r="D6">
-        <v>-0.3443752846536765</v>
-      </c>
-      <c r="E6">
-        <v>-0.2134109042609104</v>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Zona rural</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>urbano</t>
-        </is>
-      </c>
-      <c r="B7">
-        <v>-0.2220607254316475</v>
-      </c>
-      <c r="C7">
-        <v>0.01841878918019367</v>
-      </c>
-      <c r="D7">
-        <v>-0.2581615522248271</v>
-      </c>
-      <c r="E7">
+      <c r="E2" s="2">
+        <v>-9.4544857238379576E-2</v>
+      </c>
+      <c r="F2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="2">
+        <v>-0.12058408601466181</v>
+      </c>
+      <c r="C3" s="2">
+        <v>0.1037966112137393</v>
+      </c>
+      <c r="D3" s="2">
+        <v>-0.32402544399359079</v>
+      </c>
+      <c r="E3" s="2">
+        <v>8.2857271964267343E-2</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="2">
+        <v>-0.33868974635562132</v>
+      </c>
+      <c r="C4" s="2">
+        <v>3.6356979251560999E-2</v>
+      </c>
+      <c r="D4" s="2">
+        <v>-0.40994942568868081</v>
+      </c>
+      <c r="E4" s="2">
+        <v>-0.26743006702256172</v>
+      </c>
+      <c r="F4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="2">
+        <v>-0.40053844611214101</v>
+      </c>
+      <c r="C5" s="2">
+        <v>6.204813025641015E-2</v>
+      </c>
+      <c r="D5" s="2">
+        <v>-0.52215278141470489</v>
+      </c>
+      <c r="E5" s="2">
+        <v>-0.27892411080957707</v>
+      </c>
+      <c r="F5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" s="2">
+        <v>-0.28490979428472918</v>
+      </c>
+      <c r="C6" s="2">
+        <v>3.9538286129857568E-2</v>
+      </c>
+      <c r="D6" s="2">
+        <v>-0.36240483509924998</v>
+      </c>
+      <c r="E6" s="2">
+        <v>-0.20741475347020841</v>
+      </c>
+      <c r="F6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7" s="2">
+        <v>-0.35141826889864569</v>
+      </c>
+      <c r="C7" s="2">
+        <v>9.0342484155832847E-2</v>
+      </c>
+      <c r="D7" s="2">
+        <v>-0.52848953784407804</v>
+      </c>
+      <c r="E7" s="2">
+        <v>-0.17434699995321329</v>
+      </c>
+      <c r="F7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" s="2">
+        <v>-0.27391662566472819</v>
+      </c>
+      <c r="C8" s="2">
+        <v>9.2906312093382071E-2</v>
+      </c>
+      <c r="D8" s="2">
+        <v>-0.45601299736775702</v>
+      </c>
+      <c r="E8" s="2">
+        <v>-9.1820253961699322E-2</v>
+      </c>
+      <c r="F8" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" s="2">
+        <v>-0.18250921775362769</v>
+      </c>
+      <c r="C9" s="2">
+        <v>2.6680848030003701E-2</v>
+      </c>
+      <c r="D9" s="2">
+        <v>-0.234803679892435</v>
+      </c>
+      <c r="E9" s="2">
+        <v>-0.13021475561482049</v>
+      </c>
+      <c r="F9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>22</v>
+      </c>
+      <c r="B10" s="2">
+        <v>-0.27889309445729338</v>
+      </c>
+      <c r="C10" s="2">
+        <v>3.3409280712440349E-2</v>
+      </c>
+      <c r="D10" s="2">
+        <v>-0.34437528465367651</v>
+      </c>
+      <c r="E10" s="2">
+        <v>-0.21341090426091039</v>
+      </c>
+      <c r="F10" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>24</v>
+      </c>
+      <c r="B11" s="2">
+        <v>-0.22206072543164751</v>
+      </c>
+      <c r="C11" s="2">
+        <v>1.841878918019367E-2</v>
+      </c>
+      <c r="D11" s="2">
+        <v>-0.25816155222482712</v>
+      </c>
+      <c r="E11" s="2">
         <v>-0.1859598986384679</v>
       </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Zona urbana</t>
-        </is>
+      <c r="F11" t="s">
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>